<commit_message>
edited 7.12 to include more practice details
</commit_message>
<xml_diff>
--- a/配图和其他.xlsx
+++ b/配图和其他.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-20.04\home\timathon\codes\vexiq2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B4525AE-3EC8-4B4D-857E-1E9FF4D35C71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1612BE72-F407-4164-BF2F-92FBE18615D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="45">
   <si>
     <t>草图要真实手画的</t>
   </si>
@@ -52,9 +52,6 @@
     <t>p77多有模块要有注释，表明做什么，孩子必须对模块懂</t>
   </si>
   <si>
-    <t>训练过程，要有记录，多少分、策略</t>
-  </si>
-  <si>
     <t>#</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -64,10 +61,6 @@
   </si>
   <si>
     <t>具体操作</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>拍照展示底盘搭建过程，框架组合-&gt;安装车轮-&gt;安装齿轮组-&gt;安装电机-&gt;通电测试</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -136,24 +129,79 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>1）去除图片的pdf文件已生成，需要打印背景并抄写文字；
+    <t>1）已生成去除图片的pdf文件，需要打印背景并抄写文字；
 也可以不打印/抄写，直接用手绘图覆盖原有图片。
 2）草图需要手绘，草图尺寸与原图相当，之后粘贴。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>项目1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>项目2</t>
+  </si>
+  <si>
+    <t>项目3</t>
+  </si>
+  <si>
+    <t>项目4</t>
+  </si>
+  <si>
+    <t>项目5</t>
+  </si>
+  <si>
+    <t>项目6</t>
+  </si>
+  <si>
+    <t>项目7</t>
+  </si>
+  <si>
+    <t>项目8</t>
+  </si>
+  <si>
+    <t>项目9</t>
+  </si>
+  <si>
+    <t>1）已生成对应pdf文件，需要打印；
+2）然后剪下3幅小图片，粘贴到现有4.3页面内。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1）已生成对应pdf文件，需要打印；
+2）然后剪下3幅小图片，粘贴到现有P69页面内。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>难度</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1）需要老师指导添加注释
+2）抄写注释到原有页面内</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>拍照展示底盘搭建过程，比如：框架组合-&gt;安装车轮-&gt;安装齿轮组-&gt;安装电机-&gt;通电测试</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>训练过程，要有记录，多少分、策略</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>结合“训练记录”2025年10月11日-12日记录，改写“7.12 赛前集训与检查”</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1）已生成草稿；
+2）需要打印背景，并抄写文字。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>1）需要照片；
 2）而后根据照片排版，
-3）再打印并抄写。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>将原有“6.4 模拟实战：团队配合演练”章节变为“6.4.2"；
-增加"6.4.1 模拟实战：训练记录”</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>1）已生成草稿；</t>
+3）再打印背景并抄写。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -185,7 +233,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -193,14 +241,33 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -482,175 +549,214 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="2.625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.25" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="52.75" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="75.25" customWidth="1"/>
     <col min="5" max="5" width="44.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="71.25" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="3">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F2" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="42.75" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F3" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="28.5" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="3">
+        <v>3.4</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" s="3">
+        <v>3.4</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="28.5" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="3">
+        <v>4.3</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="71.25" x14ac:dyDescent="0.2">
-      <c r="A2">
+      <c r="E6" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F6" s="1">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2">
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="3">
         <v>4.4000000000000004</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="42.75" x14ac:dyDescent="0.2">
-      <c r="A3">
+      <c r="D7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F7" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="28.5" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" s="3">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="F8" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="28.5" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" s="3">
+        <v>5.5</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F9" s="1">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="28.5" x14ac:dyDescent="0.2">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
+    </row>
+    <row r="10" spans="1:6" ht="28.5" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C10" s="3">
+        <v>7.12</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="F10" s="1">
         <v>2</v>
-      </c>
-      <c r="C4">
-        <v>3.4</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
-        <v>3</v>
-      </c>
-      <c r="C5">
-        <v>3.4</v>
-      </c>
-      <c r="D5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6">
-        <v>4.3</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" t="s">
-        <v>5</v>
-      </c>
-      <c r="C7">
-        <v>4.4000000000000004</v>
-      </c>
-      <c r="D7" t="s">
-        <v>25</v>
-      </c>
-      <c r="E7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="s">
-        <v>6</v>
-      </c>
-      <c r="C8">
-        <v>4.4000000000000004</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="s">
-        <v>7</v>
-      </c>
-      <c r="C9">
-        <v>5.5</v>
-      </c>
-      <c r="D9" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="28.5" x14ac:dyDescent="0.2">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" t="s">
-        <v>8</v>
-      </c>
-      <c r="C10">
-        <v>6.4</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="E10" t="s">
-        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -669,13 +775,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -686,7 +792,7 @@
         <v>3.4</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>